<commit_message>
Repeat qPCR of the second-step PCR (SI 9, SI 10) with the corrected primer
The first qPCR used a wrongly designed primer. The qPCR was repeated with all five amplicon pools at the
same template amount (10^6 copies per reaction, 18 replicates per taxon), including a melt curve analysis
and a gel to check the amplicon size.

- SI 10: new raw data, per-well efficiencies, new sheet "Melt curves" and column "Melt peaks (n)"
- SI 9: new methods, results, Figure 9.1 (now with melt curves, panel C) and Table 9.1
- script: supporting_information_9_1 adds panel C (melt curves); results unchanged otherwise
- README and overview: mention of the melt curves

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supporting information/supporting information 9_2.xlsx
+++ b/supporting information/supporting information 9_2.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dominik\Desktop\NextCloud_lokal\QMB\01_new_submission\supporting information\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC371759-0DCC-4860-B70A-0021CDDF60C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43485" yWindow="1320" windowWidth="25365" windowHeight="19530" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -52,8 +46,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,25 +106,17 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -168,7 +154,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -202,7 +188,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -237,10 +222,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -413,16 +397,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11.28515625" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -436,74 +415,74 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>4</v>
       </c>
       <c r="B2">
-        <v>1.923</v>
+        <v>1.824</v>
       </c>
       <c r="C2">
-        <v>1.847</v>
+        <v>1.785</v>
       </c>
       <c r="D2">
-        <v>2.016</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1.872</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3">
-        <v>1.9259999999999999</v>
+        <v>1.808</v>
       </c>
       <c r="C3">
-        <v>1.8939999999999999</v>
+        <v>1.785</v>
       </c>
       <c r="D3">
-        <v>1.968</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1.834</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4">
-        <v>1.9419999999999999</v>
+        <v>1.812</v>
       </c>
       <c r="C4">
-        <v>1.917</v>
+        <v>1.793</v>
       </c>
       <c r="D4">
-        <v>1.972</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1.828</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5">
-        <v>1.9330000000000001</v>
+        <v>1.815</v>
       </c>
       <c r="C5">
-        <v>1.86</v>
+        <v>1.784</v>
       </c>
       <c r="D5">
-        <v>1.9590000000000001</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1.842</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" t="s">
         <v>8</v>
       </c>
       <c r="B6">
-        <v>1.9279999999999999</v>
+        <v>1.811</v>
       </c>
       <c r="C6">
-        <v>1.899</v>
+        <v>1.772</v>
       </c>
       <c r="D6">
-        <v>1.974</v>
+        <v>1.858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>